<commit_message>
fix(epirank): correct metadata mode in EpiRank_改 export and refresh seqday result
</commit_message>
<xml_diff>
--- a/EpiRank_改/ERA_result_seqday_d_0.95_loops_116.xlsx
+++ b/EpiRank_改/ERA_result_seqday_d_0.95_loops_116.xlsx
@@ -1179,10 +1179,10 @@
         <v>0.012838</v>
       </c>
       <c r="Y5" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z5" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="3" t="n">
         <v>11</v>
@@ -1485,10 +1485,10 @@
         <v>0.009434</v>
       </c>
       <c r="Y7" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z7" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA7" s="3" t="n">
         <v>2</v>
@@ -2403,10 +2403,10 @@
         <v>0.004698</v>
       </c>
       <c r="Y13" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z13" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA13" s="3" t="n">
         <v>4</v>
@@ -3008,7 +3008,7 @@
         <v>0.008274999999999999</v>
       </c>
       <c r="Y17" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z17" s="3" t="n">
         <v>0</v>
@@ -4228,10 +4228,10 @@
         <v>0.005408</v>
       </c>
       <c r="Y26" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z26" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA26" s="3" t="n">
         <v>7</v>
@@ -4488,10 +4488,10 @@
         <v>0.007023</v>
       </c>
       <c r="Y28" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z28" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA28" s="3" t="n">
         <v>8</v>
@@ -5231,7 +5231,7 @@
         <v>0</v>
       </c>
       <c r="Z34" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA34" s="3" t="n">
         <v>4</v>
@@ -6188,10 +6188,10 @@
         <v>0.01038</v>
       </c>
       <c r="Y42" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z42" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA42" s="3" t="n">
         <v>0</v>
@@ -6668,10 +6668,10 @@
         <v>0.005831</v>
       </c>
       <c r="Y46" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z46" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA46" s="3" t="n">
         <v>0</v>
@@ -7028,10 +7028,10 @@
         <v>0.006149</v>
       </c>
       <c r="Y49" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z49" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA49" s="3" t="n">
         <v>5</v>
@@ -7148,7 +7148,7 @@
         <v>0.004587</v>
       </c>
       <c r="Y50" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z50" s="3" t="n">
         <v>-0</v>
@@ -7988,10 +7988,10 @@
         <v>0.005555</v>
       </c>
       <c r="Y57" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z57" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA57" s="3" t="n">
         <v>2</v>
@@ -9548,7 +9548,7 @@
         <v>0.004618</v>
       </c>
       <c r="Y70" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z70" s="3" t="n">
         <v>-0</v>
@@ -9658,7 +9658,7 @@
         <v>0.002491</v>
       </c>
       <c r="Y71" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z71" s="3" t="n">
         <v>-0</v>
@@ -11088,7 +11088,7 @@
         <v>0.002498</v>
       </c>
       <c r="Y84" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z84" s="3" t="n">
         <v>0</v>
@@ -11418,7 +11418,7 @@
         <v>0.003041</v>
       </c>
       <c r="Y87" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z87" s="3" t="n">
         <v>-0</v>
@@ -11861,7 +11861,7 @@
         <v>0</v>
       </c>
       <c r="Z91" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA91" s="3" t="n">
         <v>2</v>
@@ -11968,10 +11968,10 @@
         <v>0.004355</v>
       </c>
       <c r="Y92" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z92" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA92" s="3" t="n">
         <v>0</v>
@@ -12078,10 +12078,10 @@
         <v>0.001988</v>
       </c>
       <c r="Y93" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z93" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA93" s="3" t="n">
         <v>2</v>
@@ -12518,10 +12518,10 @@
         <v>0.002789</v>
       </c>
       <c r="Y97" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z97" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA97" s="3" t="n">
         <v>1</v>
@@ -13071,7 +13071,7 @@
         <v>0</v>
       </c>
       <c r="Z102" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA102" s="3" t="n">
         <v>0</v>
@@ -13288,10 +13288,10 @@
         <v>0.003369</v>
       </c>
       <c r="Y104" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z104" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA104" s="3" t="n">
         <v>2</v>
@@ -13398,10 +13398,10 @@
         <v>0.003781</v>
       </c>
       <c r="Y105" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z105" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA105" s="3" t="n">
         <v>0</v>
@@ -13621,7 +13621,7 @@
         <v>-0</v>
       </c>
       <c r="Z107" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA107" s="3" t="n">
         <v>3</v>
@@ -13728,10 +13728,10 @@
         <v>0.003716</v>
       </c>
       <c r="Y108" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z108" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA108" s="3" t="n">
         <v>0</v>
@@ -14058,10 +14058,10 @@
         <v>0.002802</v>
       </c>
       <c r="Y111" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z111" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA111" s="3" t="n">
         <v>0</v>
@@ -14168,10 +14168,10 @@
         <v>0.003672</v>
       </c>
       <c r="Y112" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z112" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA112" s="3" t="n">
         <v>0</v>
@@ -14391,7 +14391,7 @@
         <v>-0</v>
       </c>
       <c r="Z114" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA114" s="3" t="n">
         <v>1</v>
@@ -14498,10 +14498,10 @@
         <v>0.002806</v>
       </c>
       <c r="Y115" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z115" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA115" s="3" t="n">
         <v>0</v>
@@ -14718,10 +14718,10 @@
         <v>0.0059</v>
       </c>
       <c r="Y117" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z117" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA117" s="3" t="n">
         <v>0</v>
@@ -14828,10 +14828,10 @@
         <v>0.002833</v>
       </c>
       <c r="Y118" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z118" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA118" s="3" t="n">
         <v>0</v>
@@ -14938,10 +14938,10 @@
         <v>0.002833</v>
       </c>
       <c r="Y119" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z119" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA119" s="3" t="n">
         <v>1</v>
@@ -15048,10 +15048,10 @@
         <v>0.003882</v>
       </c>
       <c r="Y120" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z120" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA120" s="3" t="n">
         <v>0</v>
@@ -15158,10 +15158,10 @@
         <v>0.001286</v>
       </c>
       <c r="Y121" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z121" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA121" s="3" t="n">
         <v>1</v>
@@ -15271,7 +15271,7 @@
         <v>0</v>
       </c>
       <c r="Z122" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA122" s="3" t="n">
         <v>2</v>
@@ -15488,10 +15488,10 @@
         <v>0.001759</v>
       </c>
       <c r="Y124" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z124" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA124" s="3" t="n">
         <v>1</v>
@@ -16478,10 +16478,10 @@
         <v>0.002594</v>
       </c>
       <c r="Y133" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z133" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA133" s="3" t="n">
         <v>0</v>
@@ -16591,7 +16591,7 @@
         <v>-0</v>
       </c>
       <c r="Z134" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA134" s="3" t="n">
         <v>3</v>
@@ -16698,10 +16698,10 @@
         <v>0.002116</v>
       </c>
       <c r="Y135" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z135" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA135" s="3" t="n">
         <v>0</v>
@@ -17358,7 +17358,7 @@
         <v>0.002448</v>
       </c>
       <c r="Y141" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z141" s="3" t="n">
         <v>0</v>
@@ -17578,10 +17578,10 @@
         <v>0.00181</v>
       </c>
       <c r="Y143" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z143" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA143" s="3" t="n">
         <v>1</v>
@@ -17688,7 +17688,7 @@
         <v>0.001664</v>
       </c>
       <c r="Y144" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z144" s="3" t="n">
         <v>-0</v>
@@ -17798,10 +17798,10 @@
         <v>0.001951</v>
       </c>
       <c r="Y145" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z145" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA145" s="3" t="n">
         <v>0</v>
@@ -18678,10 +18678,10 @@
         <v>0.001714</v>
       </c>
       <c r="Y153" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z153" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA153" s="3" t="n">
         <v>2</v>
@@ -18898,10 +18898,10 @@
         <v>0.001295</v>
       </c>
       <c r="Y155" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z155" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA155" s="3" t="n">
         <v>0</v>
@@ -19008,10 +19008,10 @@
         <v>0.002578</v>
       </c>
       <c r="Y156" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z156" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA156" s="3" t="n">
         <v>0</v>
@@ -19231,7 +19231,7 @@
         <v>0</v>
       </c>
       <c r="Z158" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA158" s="3" t="n">
         <v>1</v>
@@ -19448,7 +19448,7 @@
         <v>0.002491</v>
       </c>
       <c r="Y160" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z160" s="3" t="n">
         <v>0</v>
@@ -19888,10 +19888,10 @@
         <v>0.001307</v>
       </c>
       <c r="Y164" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z164" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA164" s="3" t="n">
         <v>0</v>
@@ -20001,7 +20001,7 @@
         <v>-0</v>
       </c>
       <c r="Z165" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA165" s="3" t="n">
         <v>0</v>
@@ -20328,10 +20328,10 @@
         <v>0.004473</v>
       </c>
       <c r="Y168" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z168" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA168" s="3" t="n">
         <v>1</v>
@@ -20548,7 +20548,7 @@
         <v>0.00302</v>
       </c>
       <c r="Y170" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z170" s="3" t="n">
         <v>0</v>
@@ -20881,7 +20881,7 @@
         <v>-0</v>
       </c>
       <c r="Z173" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA173" s="3" t="n">
         <v>0</v>
@@ -21211,7 +21211,7 @@
         <v>0</v>
       </c>
       <c r="Z176" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA176" s="3" t="n">
         <v>0</v>
@@ -21321,7 +21321,7 @@
         <v>0</v>
       </c>
       <c r="Z177" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA177" s="3" t="n">
         <v>2</v>
@@ -21431,7 +21431,7 @@
         <v>0</v>
       </c>
       <c r="Z178" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA178" s="3" t="n">
         <v>0</v>
@@ -21648,10 +21648,10 @@
         <v>0.001235</v>
       </c>
       <c r="Y180" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z180" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA180" s="3" t="n">
         <v>1</v>
@@ -21758,10 +21758,10 @@
         <v>0.001797</v>
       </c>
       <c r="Y181" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z181" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA181" s="3" t="n">
         <v>0</v>
@@ -22528,10 +22528,10 @@
         <v>0.001192</v>
       </c>
       <c r="Y188" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z188" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA188" s="3" t="n">
         <v>0</v>
@@ -22748,10 +22748,10 @@
         <v>0.002542</v>
       </c>
       <c r="Y190" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z190" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA190" s="3" t="n">
         <v>1</v>
@@ -22861,7 +22861,7 @@
         <v>0</v>
       </c>
       <c r="Z191" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA191" s="3" t="n">
         <v>0</v>
@@ -22968,10 +22968,10 @@
         <v>0.001259</v>
       </c>
       <c r="Y192" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z192" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA192" s="3" t="n">
         <v>1</v>
@@ -23188,10 +23188,10 @@
         <v>0.001644</v>
       </c>
       <c r="Y194" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z194" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA194" s="3" t="n">
         <v>1</v>
@@ -23518,7 +23518,7 @@
         <v>0.002087</v>
       </c>
       <c r="Y197" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z197" s="3" t="n">
         <v>-0</v>
@@ -23848,10 +23848,10 @@
         <v>0.002818</v>
       </c>
       <c r="Y200" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z200" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA200" s="3" t="n">
         <v>0</v>
@@ -23958,10 +23958,10 @@
         <v>0.002161</v>
       </c>
       <c r="Y201" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z201" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA201" s="3" t="n">
         <v>0</v>
@@ -24291,7 +24291,7 @@
         <v>-0</v>
       </c>
       <c r="Z204" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA204" s="3" t="n">
         <v>6</v>
@@ -24401,7 +24401,7 @@
         <v>0</v>
       </c>
       <c r="Z205" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA205" s="3" t="n">
         <v>0</v>
@@ -24511,7 +24511,7 @@
         <v>0</v>
       </c>
       <c r="Z206" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA206" s="3" t="n">
         <v>1</v>
@@ -24728,10 +24728,10 @@
         <v>0.001245</v>
       </c>
       <c r="Y208" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z208" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA208" s="3" t="n">
         <v>0</v>
@@ -24951,7 +24951,7 @@
         <v>0</v>
       </c>
       <c r="Z210" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA210" s="3" t="n">
         <v>1</v>
@@ -25608,10 +25608,10 @@
         <v>0.001782</v>
       </c>
       <c r="Y216" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z216" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z216" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA216" s="3" t="n">
         <v>2</v>
@@ -26161,7 +26161,7 @@
         <v>0</v>
       </c>
       <c r="Z221" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA221" s="3" t="n">
         <v>2</v>
@@ -26268,7 +26268,7 @@
         <v>0.001</v>
       </c>
       <c r="Y222" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z222" s="3" t="n">
         <v>0</v>
@@ -26381,7 +26381,7 @@
         <v>0</v>
       </c>
       <c r="Z223" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA223" s="3" t="n">
         <v>2</v>
@@ -26788,7 +26788,7 @@
         <v>0.000905</v>
       </c>
       <c r="Y227" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z227" s="3" t="n">
         <v>0</v>
@@ -26891,7 +26891,7 @@
         <v>0</v>
       </c>
       <c r="Z228" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA228" s="3" t="n">
         <v>3</v>
@@ -27088,7 +27088,7 @@
         <v>0.000867</v>
       </c>
       <c r="Y230" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z230" s="3" t="n">
         <v>-0</v>
@@ -27188,10 +27188,10 @@
         <v>0.00135</v>
       </c>
       <c r="Y231" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z231" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA231" s="3" t="n">
         <v>0</v>
@@ -27288,7 +27288,7 @@
         <v>0.00185</v>
       </c>
       <c r="Y232" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z232" s="3" t="n">
         <v>-0</v>
@@ -27388,10 +27388,10 @@
         <v>0.001386</v>
       </c>
       <c r="Y233" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z233" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA233" s="3" t="n">
         <v>0</v>
@@ -27488,7 +27488,7 @@
         <v>0.001592</v>
       </c>
       <c r="Y234" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z234" s="3" t="n">
         <v>-0</v>
@@ -27591,7 +27591,7 @@
         <v>-0</v>
       </c>
       <c r="Z235" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA235" s="3" t="n">
         <v>0</v>
@@ -27888,7 +27888,7 @@
         <v>0.000672</v>
       </c>
       <c r="Y238" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z238" s="3" t="n">
         <v>-0</v>
@@ -28088,10 +28088,10 @@
         <v>0.00144</v>
       </c>
       <c r="Y240" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z240" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA240" s="3" t="n">
         <v>0</v>
@@ -28288,10 +28288,10 @@
         <v>0.002059</v>
       </c>
       <c r="Y242" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z242" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA242" s="3" t="n">
         <v>0</v>
@@ -28491,7 +28491,7 @@
         <v>0</v>
       </c>
       <c r="Z244" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA244" s="3" t="n">
         <v>1</v>
@@ -28688,7 +28688,7 @@
         <v>0.001248</v>
       </c>
       <c r="Y246" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z246" s="3" t="n">
         <v>-0</v>
@@ -28888,7 +28888,7 @@
         <v>0.001999</v>
       </c>
       <c r="Y248" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z248" s="3" t="n">
         <v>-0</v>
@@ -29088,7 +29088,7 @@
         <v>0.001577</v>
       </c>
       <c r="Y250" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z250" s="3" t="n">
         <v>-0</v>
@@ -29288,7 +29288,7 @@
         <v>0.001036</v>
       </c>
       <c r="Y252" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z252" s="3" t="n">
         <v>-0</v>
@@ -29388,10 +29388,10 @@
         <v>0.001663</v>
       </c>
       <c r="Y253" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z253" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA253" s="3" t="n">
         <v>0</v>
@@ -29688,10 +29688,10 @@
         <v>0.001513</v>
       </c>
       <c r="Y256" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z256" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA256" s="3" t="n">
         <v>3</v>
@@ -29988,10 +29988,10 @@
         <v>0.00209</v>
       </c>
       <c r="Y259" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z259" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA259" s="3" t="n">
         <v>1</v>
@@ -30291,7 +30291,7 @@
         <v>-0</v>
       </c>
       <c r="Z262" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA262" s="3" t="n">
         <v>0</v>
@@ -30391,7 +30391,7 @@
         <v>-0</v>
       </c>
       <c r="Z263" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA263" s="3" t="n">
         <v>0</v>
@@ -31588,7 +31588,7 @@
         <v>0.000804</v>
       </c>
       <c r="Y275" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z275" s="3" t="n">
         <v>0</v>
@@ -32188,10 +32188,10 @@
         <v>0.00087</v>
       </c>
       <c r="Y281" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z281" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA281" s="3" t="n">
         <v>1</v>
@@ -32388,7 +32388,7 @@
         <v>0.000883</v>
       </c>
       <c r="Y283" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z283" s="3" t="n">
         <v>-0</v>
@@ -32491,7 +32491,7 @@
         <v>-0</v>
       </c>
       <c r="Z284" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA284" s="3" t="n">
         <v>0</v>
@@ -32788,7 +32788,7 @@
         <v>0.00315</v>
       </c>
       <c r="Y287" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z287" s="3" t="n">
         <v>-0</v>
@@ -33388,10 +33388,10 @@
         <v>0.001773</v>
       </c>
       <c r="Y293" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z293" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z293" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA293" s="3" t="n">
         <v>1</v>
@@ -33491,7 +33491,7 @@
         <v>0</v>
       </c>
       <c r="Z294" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA294" s="3" t="n">
         <v>1</v>
@@ -33791,7 +33791,7 @@
         <v>0</v>
       </c>
       <c r="Z297" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA297" s="3" t="n">
         <v>0</v>
@@ -33891,7 +33891,7 @@
         <v>0</v>
       </c>
       <c r="Z298" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA298" s="3" t="n">
         <v>2</v>
@@ -34391,7 +34391,7 @@
         <v>0</v>
       </c>
       <c r="Z303" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA303" s="3" t="n">
         <v>0</v>
@@ -34491,7 +34491,7 @@
         <v>0</v>
       </c>
       <c r="Z304" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA304" s="3" t="n">
         <v>0</v>
@@ -34588,7 +34588,7 @@
         <v>0.000908</v>
       </c>
       <c r="Y305" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z305" s="3" t="n">
         <v>0</v>
@@ -35188,10 +35188,10 @@
         <v>0.000919</v>
       </c>
       <c r="Y311" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z311" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z311" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA311" s="3" t="n">
         <v>0</v>
@@ -35391,7 +35391,7 @@
         <v>-0</v>
       </c>
       <c r="Z313" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA313" s="3" t="n">
         <v>0</v>
@@ -35791,7 +35791,7 @@
         <v>0</v>
       </c>
       <c r="Z317" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA317" s="3" t="n">
         <v>1</v>
@@ -36091,7 +36091,7 @@
         <v>0</v>
       </c>
       <c r="Z320" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA320" s="3" t="n">
         <v>0</v>
@@ -36191,7 +36191,7 @@
         <v>0</v>
       </c>
       <c r="Z321" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA321" s="3" t="n">
         <v>0</v>
@@ -36388,10 +36388,10 @@
         <v>0.000819</v>
       </c>
       <c r="Y323" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z323" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA323" s="3" t="n">
         <v>3</v>
@@ -36588,7 +36588,7 @@
         <v>0.00087</v>
       </c>
       <c r="Y325" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z325" s="3" t="n">
         <v>0</v>
@@ -37188,10 +37188,10 @@
         <v>0.000763</v>
       </c>
       <c r="Y331" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z331" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z331" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA331" s="3" t="n">
         <v>0</v>
@@ -37791,7 +37791,7 @@
         <v>-0</v>
       </c>
       <c r="Z337" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA337" s="3" t="n">
         <v>0</v>
@@ -37988,10 +37988,10 @@
         <v>0.001202</v>
       </c>
       <c r="Y339" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z339" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA339" s="3" t="n">
         <v>0</v>
@@ -38388,7 +38388,7 @@
         <v>0.000725</v>
       </c>
       <c r="Y343" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z343" s="3" t="n">
         <v>0</v>
@@ -38488,10 +38488,10 @@
         <v>0.000561</v>
       </c>
       <c r="Y344" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z344" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA344" s="3" t="n">
         <v>0</v>
@@ -39564,10 +39564,10 @@
         <v>0.529801</v>
       </c>
       <c r="Y356" s="3" t="n">
-        <v>0.052166</v>
+        <v>0.085462</v>
       </c>
       <c r="Z356" s="3" t="n">
-        <v>0.106841</v>
+        <v>0.07013800000000001</v>
       </c>
       <c r="AB356" s="3" t="n">
         <v>0.636302</v>
@@ -39626,10 +39626,10 @@
         <v>0.445424</v>
       </c>
       <c r="Y358" s="3" t="n">
-        <v>0.368239</v>
+        <v>0.374105</v>
       </c>
       <c r="Z358" s="3" t="n">
-        <v>0.381881</v>
+        <v>0.360217</v>
       </c>
       <c r="AA358" s="3" t="n">
         <v>0.552812</v>
@@ -40001,10 +40001,10 @@
         <v>0.386474</v>
       </c>
       <c r="D8" t="n">
-        <v>0.368239</v>
+        <v>0.374105</v>
       </c>
       <c r="E8" t="n">
-        <v>0.281734</v>
+        <v>0.288422</v>
       </c>
       <c r="F8" t="n">
         <v>0.2988505747126437</v>
@@ -40031,10 +40031,10 @@
         <v>0.216528</v>
       </c>
       <c r="D9" t="n">
-        <v>0.052166</v>
+        <v>0.085462</v>
       </c>
       <c r="E9" t="n">
-        <v>0.039429</v>
+        <v>0.06575</v>
       </c>
       <c r="F9" t="n">
         <v>0.1641791044776119</v>
@@ -40061,10 +40061,10 @@
         <v>0.41859</v>
       </c>
       <c r="D10" t="n">
-        <v>0.332634</v>
+        <v>0.352684</v>
       </c>
       <c r="E10" t="n">
-        <v>0.270229</v>
+        <v>0.286078</v>
       </c>
       <c r="F10" t="n">
         <v>0.3636363636363636</v>
@@ -40091,10 +40091,10 @@
         <v>0.397421</v>
       </c>
       <c r="D11" t="n">
-        <v>0.381881</v>
+        <v>0.360217</v>
       </c>
       <c r="E11" t="n">
-        <v>0.285561</v>
+        <v>0.27029</v>
       </c>
       <c r="F11" t="n">
         <v>0.3333333333333333</v>
@@ -40121,10 +40121,10 @@
         <v>0.219019</v>
       </c>
       <c r="D12" t="n">
-        <v>0.106841</v>
+        <v>0.07013800000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.08237999999999999</v>
+        <v>0.053723</v>
       </c>
       <c r="F12" t="n">
         <v>0.1716417910447761</v>
@@ -40151,10 +40151,10 @@
         <v>0.43754</v>
       </c>
       <c r="D13" t="n">
-        <v>0.343323</v>
+        <v>0.355855</v>
       </c>
       <c r="E13" t="n">
-        <v>0.27947</v>
+        <v>0.288879</v>
       </c>
       <c r="F13" t="n">
         <v>0.3939393939393939</v>

</xml_diff>